<commit_message>
fix: bold statement, SM/Product batch logic, TEST field dynamic
</commit_message>
<xml_diff>
--- a/api/AMV_report.xlsx
+++ b/api/AMV_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Automation\Project Automation CTD\mvr-live\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C0B01B-DBDE-4C36-8DDF-B3F63AD9D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A3D3FD-AFF7-4FC5-8BB6-1CB38B3FE2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -282,9 +282,6 @@
     <t>Conc (mg/ml)</t>
   </si>
   <si>
-    <t>Avanafil 200mg Tablets</t>
-  </si>
-  <si>
     <t>Test</t>
   </si>
   <si>
@@ -306,10 +303,13 @@
     <t>QC-195</t>
   </si>
   <si>
-    <t>sm</t>
-  </si>
-  <si>
-    <t>balafil</t>
+    <t>p</t>
+  </si>
+  <si>
+    <t>sildenafil</t>
+  </si>
+  <si>
+    <t>Tadalafil 200mg Tablets</t>
   </si>
 </sst>
 </file>
@@ -544,9 +544,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -555,6 +552,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1251,15 +1251,15 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1267,7 +1267,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1280,16 +1280,16 @@
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" s="2"/>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1305,32 +1305,36 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" s="2">
         <v>1546</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
-        <v>86</v>
+      <c r="A11" s="22" t="s">
+        <v>85</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="24"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="23"/>
+      <c r="B12" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="25"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="2">
+        <v>5</v>
+      </c>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -1381,16 +1385,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">

</xml_diff>